<commit_message>
Document approximate text capacities and add template entry guidance
</commit_message>
<xml_diff>
--- a/templates/all_options_input_template.xlsx
+++ b/templates/all_options_input_template.xlsx
@@ -129,6 +129,226 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pittacia Insectorum</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with StateProv and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and StateProv; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 2 by itself. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with Verbatim_Date and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with elevation and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 5. Spaces after initials are removed for display. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with microhabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with macrohabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pittacia Insectorum</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with StateProv and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and StateProv; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 2 by itself. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with Verbatim_Date and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with elevation and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 5. Spaces after initials are removed for display. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with microhabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with macrohabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pittacia Insectorum</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with StateProv and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and StateProv; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 2 by itself. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with Verbatim_Date and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with elevation and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 5. Spaces after initials are removed for display. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with microhabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with macrohabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Pittacia Insectorum</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with StateProv and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and County; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 1 with Country and StateProv; count punctuation/spaces too. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 2 by itself. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with Verbatim_Date and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 4 with elevation and a comma/space. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Uses line 5. Spaces after initials are removed for display. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with microhabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Normal-layout length guidance (not a restriction): Arial roughly 20–23 characters at 4 pt or 23–25 at 3.5 pt per full line, including spaces/punctuation. Width varies with letters. Shares line 6 with macrohabitat at 3.5 pt; may have less room near Field Number. Separate-habitat mode has different limits. See docs/text_length_guidance.md and check the generated PDF/report.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -421,7 +641,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -513,6 +733,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -523,7 +744,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -615,6 +836,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -625,7 +847,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -717,6 +939,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -727,7 +950,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -825,6 +1048,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -835,7 +1059,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
   </cols>
@@ -859,7 +1083,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
@@ -907,7 +1131,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
   </cols>
@@ -931,7 +1155,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="65" customWidth="1" min="2" max="2"/>

</xml_diff>